<commit_message>
feat(data): move topic visuals into catalog
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ASIGNATURAS'!$A$1:$O$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TEMAS'!$A$1:$P$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TEMAS'!$A$1:$R$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MIGRACIÓN_TEMAS'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TIPOS_ACTIVIDAD'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PLATAFORMAS'!$A$1:$E$3</definedName>
@@ -797,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -807,15 +807,17 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="65" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="65" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -856,45 +858,55 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Color principal</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Color suave</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Imagen</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Texto alternativo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Posición de imagen</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ID de crédito</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ID legado</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Nombre original</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Curso histórico</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Conteo declarado legado</t>
         </is>
@@ -932,45 +944,55 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>#285F79</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>#DFEAF0</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>/sections/historia.webp</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Biblia antigua, brújula y mapa histórico sobre una mesa</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>center 58%</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-001</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>SEC-01</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Tema de la Historia (el tema de la Edad Contemporánea de 6º PRIMARIA)</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="R2" s="2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1006,41 +1028,51 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>#4F722B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>#E6EFD9</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>/sections/alimentacion.webp</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Platos con verduras, legumbres, frutos secos y otros alimentos</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-002</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>SEC-02</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>TEMA DE LA ALIMENTACIÓN (NO SÉ DE QUÉ CURSO SON LAS ACTIVIDADES)</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Curso de origen desconocido</t>
         </is>
       </c>
-      <c r="P3" s="2" t="n">
+      <c r="R3" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1076,41 +1108,51 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>#72549A</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>#ECE5F3</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>/sections/politica-y-organizacion-de-espana.webp</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Una persona deposita un sobre en una urna ante la bandera de España</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-003</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>SEC-03</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>POLÍTICA GENERAL Y ORGANIZACIÓN DE ESPAÑA (4, 5 y 6 de primaria)</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>4.º, 5.º y 6.º de Primaria</t>
         </is>
       </c>
-      <c r="P4" s="2" t="n">
+      <c r="R4" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1146,41 +1188,51 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>#A35145</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>#F3E3DE</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>/sections/sociedad-y-poblacion.webp</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Figuras de personas distribuidas sobre un mapa de Europa</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-004</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>SEC-04</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>SOCIEDAD (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="R5" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1216,41 +1268,51 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
+          <t>#1E725E</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>#D9EEE7</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>/sections/medio-ambiente-y-sostenibilidad.webp</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Manos sostienen símbolos de la Tierra, el agua, la energía y las plantas</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-005</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>SEC-05</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>MEDIO AMBIENTE Y DEMÁS (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="R6" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1282,45 +1344,55 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
+          <t>#946128</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>#F2E8D6</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>/sections/la-transicion-espanola.webp</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Proclamación de Juan Carlos I como rey de España en 1975</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>center 38%</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-006</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>SEC-06</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>LA TRANSICIÓN (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="R7" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1352,45 +1424,55 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>#3567A1</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>#DDE9F5</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>/sections/derechos-y-deberes.webp</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Puños alzados de distintos tonos de piel como símbolo de igualdad</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>center 50%</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-007</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>SEC-07</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>DERECHOS Y DEBERES (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P8" s="2" t="n">
+      <c r="R8" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1422,41 +1504,51 @@
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
+          <t>#296B88</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>#DCECF2</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>/sections/union-europea.webp</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Estrellas de la bandera de la Unión Europea sobre un mapa de Europa</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-008</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>SEC-08</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>LA UNIÓN EUROPEA (5 Y 6 DE PRIMARIA)</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>5.º y 6.º de Primaria</t>
         </is>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="R9" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1488,41 +1580,51 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
+          <t>#A14468</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>#F3DFE7</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>/sections/reproduccion-humana.webp</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Ilustración científica de espermatozoides aproximándose a un óvulo</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-009</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>SEC-09</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>LA REPRODUCCIÓN (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P10" s="2" t="n">
+      <c r="R10" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1554,45 +1656,55 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>#8B5741</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>#EFE3DC</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
           <t>/sections/cuerpo-humano.webp</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Ilustración anatómica del esqueleto, los órganos y el sistema circulatorio</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>center 42%</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-010</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>SEC-10</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>EL CUERPO HUMANO (6 PRIMARIA)</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>6.º de Primaria</t>
         </is>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="R11" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1624,46 +1736,56 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>#376D63</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>#DFECE9</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
           <t>/sections/relieve-y-geografia.webp</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Brújula sobre un mapa físico y político de Europa</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>credit-topic-ciencias-011</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>SEC-11</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>RELIEVE Y GEOGRAFÍA (4, 5 Y 6 DE PRIMARIA)</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>4.º, 5.º y 6.º de Primaria</t>
         </is>
       </c>
-      <c r="P12" s="2" t="n">
+      <c r="R12" s="2" t="n">
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P12"/>
+  <autoFilter ref="A1:R12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add approved images and credits for 21 topics
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASIGNATURAS" sheetId="1" r:id="R327e2b03203f4130"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMAS" sheetId="2" r:id="R9f10b41c31644432"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIGRACIÓN_TEMAS" sheetId="3" r:id="Rd33a52273a334a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIPOS_ACTIVIDAD" sheetId="4" r:id="R6feeb6b26d8640da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLATAFORMAS" sheetId="5" r:id="R7a44e50c769e40aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVIDADES" sheetId="6" r:id="Ra2017838b1dd427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVIDAD_TEMA" sheetId="7" r:id="R5414cf1230fe46f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRÉDITOS" sheetId="8" r:id="R94dae3ccf43a46f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTROL_DE_CALIDAD" sheetId="9" r:id="R158a302206d5446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INFORMACIÓN" sheetId="10" r:id="R425d05ee9f274c9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RECURSOS_RELACIONADOS" sheetId="11" r:id="Rb1228b4feafc4ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENTRADA_ORIGINAL" sheetId="12" r:id="R92142abc64db4f1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVISION" sheetId="13" r:id="R174f8c2b039d4d50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASIGNATURAS" sheetId="1" r:id="R6ab875326f8e44f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMAS" sheetId="2" r:id="R66c3d32aaa6f413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIGRACIÓN_TEMAS" sheetId="3" r:id="Rbfcbd9c792d54262"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIPOS_ACTIVIDAD" sheetId="4" r:id="Rd7f6c1a91a2d4729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLATAFORMAS" sheetId="5" r:id="R7df7f4f04a6e4da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVIDADES" sheetId="6" r:id="R0f96c08a528b41e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIVIDAD_TEMA" sheetId="7" r:id="R3c0461a136714695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRÉDITOS" sheetId="8" r:id="R2778061474d84a56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTROL_DE_CALIDAD" sheetId="9" r:id="Rc40bc1ee331d49b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INFORMACIÓN" sheetId="10" r:id="Rdae4d0d0c4d04e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RECURSOS_RELACIONADOS" sheetId="11" r:id="R7e4b01e2db32417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENTRADA_ORIGINAL" sheetId="12" r:id="Rdedb75fb7d9340a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVISION" sheetId="13" r:id="Rd43d383e12e545ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1478,6 +1478,8 @@
     <x:col min="16" max="16" width="65" customWidth="1"/>
     <x:col min="17" max="17" width="24" customWidth="1"/>
     <x:col min="18" max="18" width="20" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1571,6 +1573,12 @@
           <x:t xml:space="preserve">Conteo declarado legado</x:t>
         </x:is>
       </x:c>
+      <x:c r="S1" t="str">
+        <x:v>Icono</x:v>
+      </x:c>
+      <x:c r="T1" t="str">
+        <x:v>Presentación de cabecera</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="inlineStr">
@@ -2560,10 +2568,14 @@
       <x:c r="G13"/>
       <x:c r="H13"/>
       <x:c r="I13"/>
-      <x:c r="J13"/>
+      <x:c r="J13" t="str">
+        <x:v>/images/topics/topic-frances-material-escolar.webp</x:v>
+      </x:c>
       <x:c r="K13"/>
       <x:c r="L13"/>
-      <x:c r="M13"/>
+      <x:c r="M13" t="str">
+        <x:v>credit-topic-frances-material-escolar</x:v>
+      </x:c>
       <x:c r="N13" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2571,6 +2583,7 @@
       <x:c r="P13"/>
       <x:c r="Q13"/>
       <x:c r="R13"/>
+      <x:c r="T13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
@@ -2592,10 +2605,14 @@
       <x:c r="G14"/>
       <x:c r="H14"/>
       <x:c r="I14"/>
-      <x:c r="J14"/>
+      <x:c r="J14" t="str">
+        <x:v>/images/topics/topic-frances-vetements.webp</x:v>
+      </x:c>
       <x:c r="K14"/>
       <x:c r="L14"/>
-      <x:c r="M14"/>
+      <x:c r="M14" t="str">
+        <x:v>credit-topic-frances-vetements</x:v>
+      </x:c>
       <x:c r="N14" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2603,6 +2620,7 @@
       <x:c r="P14"/>
       <x:c r="Q14"/>
       <x:c r="R14"/>
+      <x:c r="T14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
@@ -2624,10 +2642,16 @@
       <x:c r="G15"/>
       <x:c r="H15"/>
       <x:c r="I15"/>
-      <x:c r="J15"/>
+      <x:c r="J15" t="str">
+        <x:v>/images/topics/topic-frances-ecole.webp</x:v>
+      </x:c>
       <x:c r="K15"/>
-      <x:c r="L15"/>
-      <x:c r="M15"/>
+      <x:c r="L15" t="str">
+        <x:v>58% 43%</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>credit-topic-frances-ecole</x:v>
+      </x:c>
       <x:c r="N15" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2635,6 +2659,7 @@
       <x:c r="P15"/>
       <x:c r="Q15"/>
       <x:c r="R15"/>
+      <x:c r="T15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
@@ -2656,10 +2681,18 @@
       <x:c r="G16"/>
       <x:c r="H16"/>
       <x:c r="I16"/>
-      <x:c r="J16"/>
-      <x:c r="K16"/>
-      <x:c r="L16"/>
-      <x:c r="M16"/>
+      <x:c r="J16" t="str">
+        <x:v>/images/topics/topic-frances-prepositions-lieu.webp</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>Una pelota está encima, debajo y al lado de tres sillas.</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>50% 46%</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>credit-topic-frances-prepositions-lieu</x:v>
+      </x:c>
       <x:c r="N16" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2667,6 +2700,7 @@
       <x:c r="P16"/>
       <x:c r="Q16"/>
       <x:c r="R16"/>
+      <x:c r="T16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
@@ -2688,10 +2722,16 @@
       <x:c r="G17"/>
       <x:c r="H17"/>
       <x:c r="I17"/>
-      <x:c r="J17"/>
+      <x:c r="J17" t="str">
+        <x:v>/images/topics/topic-frances-heure.webp</x:v>
+      </x:c>
       <x:c r="K17"/>
-      <x:c r="L17"/>
-      <x:c r="M17"/>
+      <x:c r="L17" t="str">
+        <x:v>72% 40%</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>credit-topic-frances-heure</x:v>
+      </x:c>
       <x:c r="N17" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2699,6 +2739,7 @@
       <x:c r="P17"/>
       <x:c r="Q17"/>
       <x:c r="R17"/>
+      <x:c r="T17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
@@ -2720,10 +2761,16 @@
       <x:c r="G18"/>
       <x:c r="H18"/>
       <x:c r="I18"/>
-      <x:c r="J18"/>
-      <x:c r="K18"/>
+      <x:c r="J18" t="str">
+        <x:v>/images/topics/topic-frances-verbes-present.webp</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>Tres escenas relacionan las acciones con «je vais», «tu joues» e «il fait».</x:v>
+      </x:c>
       <x:c r="L18"/>
-      <x:c r="M18"/>
+      <x:c r="M18" t="str">
+        <x:v>credit-topic-frances-verbes-present</x:v>
+      </x:c>
       <x:c r="N18" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2731,6 +2778,7 @@
       <x:c r="P18"/>
       <x:c r="Q18"/>
       <x:c r="R18"/>
+      <x:c r="T18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
@@ -2752,10 +2800,14 @@
       <x:c r="G19"/>
       <x:c r="H19"/>
       <x:c r="I19"/>
-      <x:c r="J19"/>
+      <x:c r="J19" t="str">
+        <x:v>/images/topics/topic-frances-loisirs.webp</x:v>
+      </x:c>
       <x:c r="K19"/>
       <x:c r="L19"/>
-      <x:c r="M19"/>
+      <x:c r="M19" t="str">
+        <x:v>credit-topic-frances-loisirs</x:v>
+      </x:c>
       <x:c r="N19" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2763,6 +2815,7 @@
       <x:c r="P19"/>
       <x:c r="Q19"/>
       <x:c r="R19"/>
+      <x:c r="T19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
@@ -2784,10 +2837,16 @@
       <x:c r="G20"/>
       <x:c r="H20"/>
       <x:c r="I20"/>
-      <x:c r="J20"/>
+      <x:c r="J20" t="str">
+        <x:v>/images/topics/topic-frances-maison.webp</x:v>
+      </x:c>
       <x:c r="K20"/>
-      <x:c r="L20"/>
-      <x:c r="M20"/>
+      <x:c r="L20" t="str">
+        <x:v>54% 48%</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>credit-topic-frances-maison</x:v>
+      </x:c>
       <x:c r="N20" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2795,6 +2854,9 @@
       <x:c r="P20"/>
       <x:c r="Q20"/>
       <x:c r="R20"/>
+      <x:c r="T20" t="str">
+        <x:v>contain</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
@@ -2816,10 +2878,14 @@
       <x:c r="G21"/>
       <x:c r="H21"/>
       <x:c r="I21"/>
-      <x:c r="J21"/>
+      <x:c r="J21" t="str">
+        <x:v>/images/topics/topic-frances-transports.webp</x:v>
+      </x:c>
       <x:c r="K21"/>
       <x:c r="L21"/>
-      <x:c r="M21"/>
+      <x:c r="M21" t="str">
+        <x:v>credit-topic-frances-transports</x:v>
+      </x:c>
       <x:c r="N21" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2827,6 +2893,7 @@
       <x:c r="P21"/>
       <x:c r="Q21"/>
       <x:c r="R21"/>
+      <x:c r="T21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
@@ -2848,10 +2915,14 @@
       <x:c r="G22"/>
       <x:c r="H22"/>
       <x:c r="I22"/>
-      <x:c r="J22"/>
+      <x:c r="J22" t="str">
+        <x:v>/images/topics/topic-frances-ville.webp</x:v>
+      </x:c>
       <x:c r="K22"/>
       <x:c r="L22"/>
-      <x:c r="M22"/>
+      <x:c r="M22" t="str">
+        <x:v>credit-topic-frances-ville</x:v>
+      </x:c>
       <x:c r="N22" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2859,6 +2930,7 @@
       <x:c r="P22"/>
       <x:c r="Q22"/>
       <x:c r="R22"/>
+      <x:c r="T22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
@@ -2880,10 +2952,16 @@
       <x:c r="G23"/>
       <x:c r="H23"/>
       <x:c r="I23"/>
-      <x:c r="J23"/>
+      <x:c r="J23" t="str">
+        <x:v>/images/topics/topic-frances-itineraires.webp</x:v>
+      </x:c>
       <x:c r="K23"/>
-      <x:c r="L23"/>
-      <x:c r="M23"/>
+      <x:c r="L23" t="str">
+        <x:v>48% 55%</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>credit-topic-frances-itineraires</x:v>
+      </x:c>
       <x:c r="N23" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2891,6 +2969,7 @@
       <x:c r="P23"/>
       <x:c r="Q23"/>
       <x:c r="R23"/>
+      <x:c r="T23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
@@ -2912,10 +2991,16 @@
       <x:c r="G24"/>
       <x:c r="H24"/>
       <x:c r="I24"/>
-      <x:c r="J24"/>
+      <x:c r="J24" t="str">
+        <x:v>/images/topics/topic-lengua-enunciados.webp</x:v>
+      </x:c>
       <x:c r="K24"/>
-      <x:c r="L24"/>
-      <x:c r="M24"/>
+      <x:c r="L24" t="str">
+        <x:v>50% 43%</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>credit-topic-lengua-enunciados</x:v>
+      </x:c>
       <x:c r="N24" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2923,6 +3008,7 @@
       <x:c r="P24"/>
       <x:c r="Q24"/>
       <x:c r="R24"/>
+      <x:c r="T24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
@@ -2944,10 +3030,14 @@
       <x:c r="G25"/>
       <x:c r="H25"/>
       <x:c r="I25"/>
-      <x:c r="J25"/>
+      <x:c r="J25" t="str">
+        <x:v>/images/topics/topic-lengua-tiempos-verbales.webp</x:v>
+      </x:c>
       <x:c r="K25"/>
       <x:c r="L25"/>
-      <x:c r="M25"/>
+      <x:c r="M25" t="str">
+        <x:v>credit-topic-lengua-tiempos-verbales</x:v>
+      </x:c>
       <x:c r="N25" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2955,6 +3045,7 @@
       <x:c r="P25"/>
       <x:c r="Q25"/>
       <x:c r="R25"/>
+      <x:c r="T25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
@@ -2976,10 +3067,14 @@
       <x:c r="G26"/>
       <x:c r="H26"/>
       <x:c r="I26"/>
-      <x:c r="J26"/>
+      <x:c r="J26" t="str">
+        <x:v>/images/topics/topic-lengua-recursos-literarios.webp</x:v>
+      </x:c>
       <x:c r="K26"/>
       <x:c r="L26"/>
-      <x:c r="M26"/>
+      <x:c r="M26" t="str">
+        <x:v>credit-topic-lengua-recursos-literarios</x:v>
+      </x:c>
       <x:c r="N26" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -2987,6 +3082,7 @@
       <x:c r="P26"/>
       <x:c r="Q26"/>
       <x:c r="R26"/>
+      <x:c r="T26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
@@ -3008,10 +3104,18 @@
       <x:c r="G27"/>
       <x:c r="H27"/>
       <x:c r="I27"/>
-      <x:c r="J27"/>
-      <x:c r="K27"/>
-      <x:c r="L27"/>
-      <x:c r="M27"/>
+      <x:c r="J27" t="str">
+        <x:v>/images/topics/topic-lengua-palabras-invariables.webp</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>La palabra con permanece igual en con niño, con niña y con niños.</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>53% 50%</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>credit-topic-lengua-palabras-invariables</x:v>
+      </x:c>
       <x:c r="N27" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3019,6 +3123,9 @@
       <x:c r="P27"/>
       <x:c r="Q27"/>
       <x:c r="R27"/>
+      <x:c r="T27" t="str">
+        <x:v>contain</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
@@ -3040,10 +3147,14 @@
       <x:c r="G28"/>
       <x:c r="H28"/>
       <x:c r="I28"/>
-      <x:c r="J28"/>
+      <x:c r="J28" t="str">
+        <x:v>/images/topics/topic-matematicas-multiplicaciones.webp</x:v>
+      </x:c>
       <x:c r="K28"/>
       <x:c r="L28"/>
-      <x:c r="M28"/>
+      <x:c r="M28" t="str">
+        <x:v>credit-topic-matematicas-multiplicaciones</x:v>
+      </x:c>
       <x:c r="N28" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3051,6 +3162,7 @@
       <x:c r="P28"/>
       <x:c r="Q28"/>
       <x:c r="R28"/>
+      <x:c r="T28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
@@ -3072,10 +3184,18 @@
       <x:c r="G29"/>
       <x:c r="H29"/>
       <x:c r="I29"/>
-      <x:c r="J29"/>
-      <x:c r="K29"/>
-      <x:c r="L29"/>
-      <x:c r="M29"/>
+      <x:c r="J29" t="str">
+        <x:v>/images/topics/topic-matematicas-rectas.webp</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>Un segmento tiene dos extremos, una semirrecta tiene un origen y las dos rectas inferiores son paralelas.</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>50% 48%</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>credit-topic-matematicas-rectas</x:v>
+      </x:c>
       <x:c r="N29" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3083,6 +3203,9 @@
       <x:c r="P29"/>
       <x:c r="Q29"/>
       <x:c r="R29"/>
+      <x:c r="T29" t="str">
+        <x:v>contain</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
@@ -3104,10 +3227,18 @@
       <x:c r="G30"/>
       <x:c r="H30"/>
       <x:c r="I30"/>
-      <x:c r="J30"/>
-      <x:c r="K30"/>
-      <x:c r="L30"/>
-      <x:c r="M30"/>
+      <x:c r="J30" t="str">
+        <x:v>/images/topics/topic-matematicas-angulos.webp</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>Tres diagramas muestran un ángulo agudo, uno recto y uno obtuso.</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>52% 52%</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>credit-topic-matematicas-angulos</x:v>
+      </x:c>
       <x:c r="N30" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3115,6 +3246,9 @@
       <x:c r="P30"/>
       <x:c r="Q30"/>
       <x:c r="R30"/>
+      <x:c r="T30" t="str">
+        <x:v>contain</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
@@ -3136,10 +3270,14 @@
       <x:c r="G31"/>
       <x:c r="H31"/>
       <x:c r="I31"/>
-      <x:c r="J31"/>
+      <x:c r="J31" t="str">
+        <x:v>/images/topics/topic-matematicas-operaciones-combinadas.webp</x:v>
+      </x:c>
       <x:c r="K31"/>
       <x:c r="L31"/>
-      <x:c r="M31"/>
+      <x:c r="M31" t="str">
+        <x:v>credit-topic-matematicas-operaciones-combinadas</x:v>
+      </x:c>
       <x:c r="N31" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3147,6 +3285,7 @@
       <x:c r="P31"/>
       <x:c r="Q31"/>
       <x:c r="R31"/>
+      <x:c r="T31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
@@ -3168,10 +3307,16 @@
       <x:c r="G32"/>
       <x:c r="H32"/>
       <x:c r="I32"/>
-      <x:c r="J32"/>
-      <x:c r="K32"/>
+      <x:c r="J32" t="str">
+        <x:v>/images/topics/topic-ingles-comparativos.webp</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>Dos plantas del mismo tipo tienen alturas diferentes.</x:v>
+      </x:c>
       <x:c r="L32"/>
-      <x:c r="M32"/>
+      <x:c r="M32" t="str">
+        <x:v>credit-topic-ingles-comparativos</x:v>
+      </x:c>
       <x:c r="N32" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3179,6 +3324,7 @@
       <x:c r="P32"/>
       <x:c r="Q32"/>
       <x:c r="R32"/>
+      <x:c r="T32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
@@ -3200,10 +3346,16 @@
       <x:c r="G33"/>
       <x:c r="H33"/>
       <x:c r="I33"/>
-      <x:c r="J33"/>
+      <x:c r="J33" t="str">
+        <x:v>/images/topics/topic-ingles-vocabulary.webp</x:v>
+      </x:c>
       <x:c r="K33"/>
-      <x:c r="L33"/>
-      <x:c r="M33"/>
+      <x:c r="L33" t="str">
+        <x:v>55% 53%</x:v>
+      </x:c>
+      <x:c r="M33" t="str">
+        <x:v>credit-topic-ingles-vocabulary</x:v>
+      </x:c>
       <x:c r="N33" t="str">
         <x:v>active</x:v>
       </x:c>
@@ -3211,6 +3363,7 @@
       <x:c r="P33"/>
       <x:c r="Q33"/>
       <x:c r="R33"/>
+      <x:c r="T33"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18781,6 +18934,468 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>credit-topic-frances-material-escolar</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Le matériel scolaire</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E13"/>
+      <x:c r="F13" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G13"/>
+      <x:c r="H13" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-material-escolar.png; SHA-256 32e63de039c6e3a5a2ab5a73bc17bdc02bc12c28b9665a0149deea932735c3a8. WebP 1600×900: b2825450e3abbbcb344ea64503584b136a3a6cea21e8504bbef0624f5aedc9b4. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>credit-topic-frances-vetements</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Les vêtements</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E14"/>
+      <x:c r="F14" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G14"/>
+      <x:c r="H14" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-vetements.png; SHA-256 978ce65c50b5f80057b13d30f0bb07e5ea0aa54ca6a7c05d0ceb166dc33df2a0. WebP 1600×900: 9b342d5ad009af786d079fb74e2f634c7ebae09c72083a6e8f1692e3dfb177ad. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>credit-topic-frances-ecole</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>L’école et les matières</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E15"/>
+      <x:c r="F15" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G15"/>
+      <x:c r="H15" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-ecole.png; SHA-256 414198423c4b6a98d18fc7800d4325c6dd14a3669bf50790a947accf7a9e9f49. WebP 1600×900: a8632b44060444ffff23418b33e083f1b4bdd19fed86f7e182c4bb47a8952ff7. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>credit-topic-frances-prepositions-lieu</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Les prépositions de lieu</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E16"/>
+      <x:c r="F16" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G16"/>
+      <x:c r="H16" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-prepositions-lieu.png; SHA-256 558720d5d48fb11fd2ca65a0cdf243e38d888fa90edd9bde31eabab2c8fa9cc2. WebP 1600×900: 6f2d333aa80c57d9c6b906d0c83bb7981ff5ba78388b0e408eb8febf0b1b0b3e. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>credit-topic-frances-heure</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>L’heure</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E17"/>
+      <x:c r="F17" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G17"/>
+      <x:c r="H17" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-heure.png; SHA-256 57bfee98d8d6d1f07c11c370ca0daf9e320b6bfbe39f8e009b07b9a97812bcaf. WebP 1600×900: 341b121ee64148004ded07947aba41566509895d6683478005f13456c4bcbbe2. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>credit-topic-frances-verbes-present</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Les verbes au présent</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E18"/>
+      <x:c r="F18" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G18"/>
+      <x:c r="H18" t="str">
+        <x:v>Generada/preparada el 2026-09-25. PNG original: topic-frances-verbes-present.png; SHA-256 98a606c9c38c108aa8aa23c1dfc86f5208893838b62befb6c719531f722e11d3. WebP 1600×900: 050f5b20808148bf8a8030e7a7fccd2b443c127e5b9826b6f8ccd28198d786e1. Archivo final recuperado: ChatGPT Image 25 sept 2026, 08_19_06 p.m..png.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>credit-topic-frances-loisirs</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Les loisirs</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E19"/>
+      <x:c r="F19" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G19"/>
+      <x:c r="H19" t="str">
+        <x:v>Generada/preparada el 2026-09-25. PNG original: topic-frances-loisirs.png; SHA-256 f7ce755becda4f99885d6cfcd35cb7f60cb495bcc9d536031aa16dfb6b724e6c. WebP 1600×900: 288c98995ed562f7a5533aa86bf476d1ed3454aeb8e0f5fa933cf00e0349415e. Archivo final recuperado: ChatGPT Image 25 sept 2026, 08_19_00 p.m..png.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>credit-topic-frances-maison</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Les pièces de la maison</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E20"/>
+      <x:c r="F20" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G20"/>
+      <x:c r="H20" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-maison.png; SHA-256 b369274543e7a09d8b799d5c89f1cc5ac008cf2baa870aab64db2c95fdfb3a86. WebP 1600×900: 7ce058d07d062da7bf5c8ada94476876de9e7348904b28b45688fa5fa8737b0d. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>credit-topic-frances-transports</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Les moyens de transport</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E21"/>
+      <x:c r="F21" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G21"/>
+      <x:c r="H21" t="str">
+        <x:v>Generada/preparada el 2026-09-25. PNG original: topic-frances-transports.png; SHA-256 5d6696a564fc0a1a875a720c441129b2e6af532961cb77f32645015989e89dc5. WebP 1600×900: 95c7d745f91ee56c64fa5d5e24967780e6c1190639daa370cbbb4d318f36af00. Archivo final recuperado: ChatGPT Image 25 sept 2026, 08_18_53 p.m..png.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>credit-topic-frances-ville</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Les lieux de la ville</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E22"/>
+      <x:c r="F22" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G22"/>
+      <x:c r="H22" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-ville.png; SHA-256 3169bb639f05d7567547b6468ff6e825a481c7e4738ef5f39a43e431da36d40b. WebP 1600×900: 654121d33c1e78c877ed371b802dc1beb5b9db6fe61f814988f30c1f817461f6. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>credit-topic-frances-itineraires</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Les itinéraires et la compréhension écrite</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E23"/>
+      <x:c r="F23" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G23"/>
+      <x:c r="H23" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-frances-itineraires.png; SHA-256 bbbb65e4336b3a7a098c8b82926f2b6b6fb37cffc8b22803bccafbefe8cae394. WebP 1600×900: 9594393de53b1d19647590bedfccf9e8dd2982607247a2a8334a319e1fa5a85b. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>credit-topic-ingles-vocabulary</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Vocabulary</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E24"/>
+      <x:c r="F24" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G24"/>
+      <x:c r="H24" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-ingles-vocabulary.png; SHA-256 8b3e909513478ddd791341991f52ef158b79c8406ebbeefe8defbd3fbd053e2d. WebP 1600×900: aa0f214ed86ecd4f3743d6a111660e91ca3767c716649e7ecf5152b4b376c24b. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>credit-topic-ingles-comparativos</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Comparative adjectives</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E25"/>
+      <x:c r="F25" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G25"/>
+      <x:c r="H25" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-ingles-comparativos.png; SHA-256 d988708afc4037e9c562aac713694018196b9ce4cb05928bd89c1f2dcd28bf33. WebP 1600×900: 3c1f71221ba87632bdb66342f54aec6c4181f3c1c7e86e3a0b99332d532c1525. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>credit-topic-lengua-enunciados</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>Tipos de enunciados</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E26"/>
+      <x:c r="F26" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G26"/>
+      <x:c r="H26" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-lengua-enunciados.png; SHA-256 2474bbed9012e8e8afb0128c1af99c2ef41a1edf465f4a21de7506c013b1148f. WebP 1600×900: 551772676be20ad5c22bbe23d42f540378a0e3a1c1829d77c4596ce7122d2a5c. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>credit-topic-lengua-tiempos-verbales</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Tiempos verbales</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E27"/>
+      <x:c r="F27" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G27"/>
+      <x:c r="H27" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-lengua-tiempos-verbales.png; SHA-256 4ea0515ed986b76b1356646e00ad04233862b8da1dd5c67846f4fd8418dd8982. WebP 1600×900: dcb626ed7a4b56df9e34e1940184b5512d4d99059707213ab0963fba39d3970c. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>credit-topic-lengua-recursos-literarios</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Recursos literarios</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E28"/>
+      <x:c r="F28" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G28"/>
+      <x:c r="H28" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-lengua-recursos-literarios.png; SHA-256 1cafa04000cec5b3e9b917650552618ef8cccf061d5ae9f85bd0a656ce55d69f. WebP 1600×900: 7623addb7ed552dd24c212d18c0834e498d7515a3309fa2d95a8585b96877f20. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>credit-topic-lengua-palabras-invariables</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Palabras invariables</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Composición y tipografía preparadas para el proyecto</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Composición local con Pillow/DejaVu Serif</x:v>
+      </x:c>
+      <x:c r="E29"/>
+      <x:c r="F29" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G29"/>
+      <x:c r="H29" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-lengua-palabras-invariables.png; SHA-256 2e639ddbfd654771f942b01e3ada2196565d7fd80a65b20d5e75515ee2ae3481. WebP 1600×900: 6075be2601c3fd4abce1bb09d4df4b4d98eeaa384390ab23458b568cac9e78d2. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>credit-topic-matematicas-multiplicaciones</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>Multiplicación</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E30"/>
+      <x:c r="F30" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G30"/>
+      <x:c r="H30" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-matematicas-multiplicaciones.png; SHA-256 6b3294210d8266b4eb46a83c85419739ab83691fae3786442aaba5b5315f1581. WebP 1600×900: 447725e59bdef74007d96fb44dd73608c5c69d8884b85832c3e37236337265c2. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>credit-topic-matematicas-rectas</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Puntos y rectas</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E31"/>
+      <x:c r="F31" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G31"/>
+      <x:c r="H31" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-matematicas-rectas.png; SHA-256 56f3c2dede09aaa9cdd57451b328cb6d85de788392a81ab6e4f87524625431ce. WebP 1600×900: a9a1b7abde25280b0a88a9962696220fb911d240754eab4f93013ece89eff4c1. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>credit-topic-matematicas-angulos</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Ángulos</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E32"/>
+      <x:c r="F32" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G32"/>
+      <x:c r="H32" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-matematicas-angulos.png; SHA-256 bcd4e1b3bf4b398229f0b7755c1bf1063d91f4d74f81a23a2777050c60fffec5. WebP 1600×900: d0626cedee54416798d428b3fd48372b57f66150e8acf71bd6140673f8133110. </x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>credit-topic-matematicas-operaciones-combinadas</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>Operaciones combinadas</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Generada con OpenAI; seleccionada por Alejandro Castaño Medina</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>ChatGPT Work (OpenAI)</x:v>
+      </x:c>
+      <x:c r="E33"/>
+      <x:c r="F33" t="str">
+        <x:v>Imagen creada para este proyecto; sin licencia externa declarada.</x:v>
+      </x:c>
+      <x:c r="G33"/>
+      <x:c r="H33" t="str">
+        <x:v>Generada/preparada el 2026-09-24. PNG original: topic-matematicas-operaciones-combinadas.png; SHA-256 1bc5bb2138465a33820974e4024a4329a1ee2a95de9eb1c969a6f04c82bd6da5. WebP 1600×900: ebf9e1625820896fd11cd5d191addb3399385fdd48bb595fecbd938366b06247. </x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
feat: redesign cell nutrition activity
</commit_message>
<xml_diff>
--- a/data/catalogo-actividades.xlsx
+++ b/data/catalogo-actividades.xlsx
@@ -17352,7 +17352,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>English-language quiz on the nutrition function in living things, including autotrophic and heterotrophic nutrition, nutrients, cellular respiration and the route oxygen follows through the body.</t>
+          <t>Interactive review of autotrophic and heterotrophic nutrition, photosynthesis and cellular respiration using labeled cell-organelle diagrams and selectable answers.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -17387,12 +17387,12 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>cellular nutrition | autotrophic nutrition | heterotrophic nutrition</t>
+          <t>cellular nutrition | photosynthesis | cellular respiration</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>nutrición celular | nutrients | cell respiration | mitochondria | oxygen pathway | nutrición autótrofa | nutrición heterótrofa</t>
+          <t>nutrición celular | autotrophic nutrition | heterotrophic nutrition | chloroplast | mitochondrion | carbon dioxide | mineral salts | oxygen | water | energy</t>
         </is>
       </c>
       <c r="P89" s="7" t="n">
@@ -17408,55 +17408,35 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>external</t>
-        </is>
-      </c>
-      <c r="T89" t="inlineStr">
-        <is>
-          <t>lumi</t>
-        </is>
-      </c>
-      <c r="U89" t="inlineStr">
-        <is>
-          <t>1PCQ0H</t>
-        </is>
-      </c>
-      <c r="V89" t="inlineStr">
+          <t>native</t>
+        </is>
+      </c>
+      <c r="X89" t="inlineStr">
         <is>
           <t>https://app.lumi.education/run/1PCQ0H</t>
         </is>
       </c>
-      <c r="W89" t="inlineStr">
-        <is>
-          <t>https://app.lumi.education/run/1PCQ0H</t>
-        </is>
-      </c>
-      <c r="X89" t="inlineStr">
-        <is>
-          <t>https://app.lumi.education/run/1PCQ0H</t>
-        </is>
-      </c>
-      <c r="Y89" t="inlineStr">
-        <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="AA89" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB89" t="inlineStr">
-        <is>
-          <t>Markdown proporcionado</t>
+      <c r="AC89" t="inlineStr">
+        <is>
+          <t>Apuntes proporcionados y recurso H5P original</t>
         </is>
       </c>
       <c r="AD89" t="inlineStr">
         <is>
-          <t>URL de origen y título proporcionados por el usuario; no verificados en navegador.</t>
-        </is>
-      </c>
-      <c r="AM89" t="inlineStr">
-        <is>
-          <t>https://app.lumi.education/run/1PCQ0H</t>
+          <t>Recurso Lumi sustituido por versión nativa; se conserva URL original para procedencia.</t>
+        </is>
+      </c>
+      <c r="AG89" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH89" t="inlineStr">
+        <is>
+          <t>mixed-practice</t>
+        </is>
+      </c>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>data/native/how-do-living-things-get-nutrients.json</t>
         </is>
       </c>
     </row>

</xml_diff>